<commit_message>
Update Global and Power Parameters in NREL-118 to newest version
</commit_message>
<xml_diff>
--- a/data/NREL-118/Global_Parameters.xlsx
+++ b/data/NREL-118/Global_Parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FelixAuer\Git\LEGO-Pyomo\data\NREL-118\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6D4F58A-4C78-4541-9592-AF6061DB65CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70CC89CB-A96B-4218-9BC4-48394CF1AFBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="851" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-4170" yWindow="-21720" windowWidth="38640" windowHeight="21120" tabRatio="851" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global Parameters" sheetId="121" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="44">
   <si>
     <t>[h]</t>
   </si>
@@ -187,6 +187,12 @@
   </si>
   <si>
     <t>Scaling factor for power values in input data (relative to 1MW)</t>
+  </si>
+  <si>
+    <t>Format:</t>
+  </si>
+  <si>
+    <t>v0.1.0</t>
   </si>
   <si>
     <t>No</t>
@@ -196,7 +202,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Calibri"/>
@@ -272,6 +278,11 @@
       <sz val="10"/>
       <name val="Aptos"/>
       <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <name val="Aptos"/>
     </font>
   </fonts>
   <fills count="8">
@@ -353,7 +364,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -402,6 +413,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
@@ -821,6 +838,14 @@
         <v>16</v>
       </c>
     </row>
+    <row r="2" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B2" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>42</v>
+      </c>
+    </row>
     <row r="3" spans="2:8" s="4" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="7" t="s">
         <v>10</v>
@@ -894,7 +919,7 @@
         <v>12</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E8" s="11" t="s">
         <v>9</v>
@@ -1233,18 +1258,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1266,6 +1291,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13778B2C-CE05-4B32-8196-2F381FEAC95A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0155F7A0-74CD-4575-8C0B-A34C113F80FE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -1279,12 +1312,4 @@
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13778B2C-CE05-4B32-8196-2F381FEAC95A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>